<commit_message>
Update management duty schedule for September 14–18
</commit_message>
<xml_diff>
--- a/grafik-dyzurow-nadzoru-2026-2027.xlsx
+++ b/grafik-dyzurow-nadzoru-2026-2027.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="grafik" sheetId="1" r:id="R22294596f56143af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="numery telefonów" sheetId="2" r:id="Rec3b4e5a11644225"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="grafik" sheetId="1" r:id="Ra2e57b67bf9a48b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="numery telefonów" sheetId="2" r:id="R4ecf62a312224c2a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -358,43 +358,81 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>08:00 - 13:30</x:v>
+        <x:v>08:00 - 10:00</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>Arkadiusz Mocarski</x:v>
-      </x:c>
-      <x:c r="C2" t="str">
-        <x:v>Arkadiusz Mocarski</x:v>
-      </x:c>
-      <x:c r="D2" t="str">
-        <x:v>Arkadiusz Mocarski</x:v>
-      </x:c>
-      <x:c r="E2" t="str">
         <x:v>Małgorzata Kończyńska</x:v>
       </x:c>
-      <x:c r="F2" t="str">
-        <x:v>Małgorzata Kończyńska</x:v>
-      </x:c>
+      <x:c r="C2" t="str"/>
+      <x:c r="D2" t="str"/>
+      <x:c r="E2" t="str"/>
+      <x:c r="F2" t="str"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>13:30 - 19:00</x:v>
-      </x:c>
-      <x:c r="B3" t="str">
-        <x:v>Wiesław Filipiak</x:v>
-      </x:c>
+        <x:v>08:00 - 13:30</x:v>
+      </x:c>
+      <x:c r="B3" t="str"/>
       <x:c r="C3" t="str">
+        <x:v>Arkadiusz Mocarski</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>Arkadiusz Mocarski</x:v>
+      </x:c>
+      <x:c r="E3" t="str">
         <x:v>Małgorzata Kończyńska</x:v>
       </x:c>
-      <x:c r="D3" t="str">
-        <x:v>Wiesław Filipiak</x:v>
-      </x:c>
-      <x:c r="E3" t="str">
-        <x:v>Wiesław Filipiak</x:v>
-      </x:c>
-      <x:c r="F3" t="str">
-        <x:v>Wiesław Filipiak</x:v>
-      </x:c>
+      <x:c r="F3" t="str"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>10:00 - 16:00</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>Maciej Najwer</x:v>
+      </x:c>
+      <x:c r="C4" t="str"/>
+      <x:c r="D4" t="str"/>
+      <x:c r="E4" t="str"/>
+      <x:c r="F4" t="str"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>13:30 - 16:00</x:v>
+      </x:c>
+      <x:c r="B5" t="str"/>
+      <x:c r="C5" t="str"/>
+      <x:c r="D5" t="str">
+        <x:v>Maciej Najwer</x:v>
+      </x:c>
+      <x:c r="E5" t="str"/>
+      <x:c r="F5" t="str"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>13:30 - 18:00</x:v>
+      </x:c>
+      <x:c r="B6" t="str"/>
+      <x:c r="C6" t="str">
+        <x:v>Małgorzata Kończyńska</x:v>
+      </x:c>
+      <x:c r="D6" t="str"/>
+      <x:c r="E6" t="str">
+        <x:v>Maciej Najwer</x:v>
+      </x:c>
+      <x:c r="F6" t="str"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>16:00 - 18:00</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>Arkadiusz Mocarski</x:v>
+      </x:c>
+      <x:c r="C7" t="str"/>
+      <x:c r="D7" t="str"/>
+      <x:c r="E7" t="str"/>
+      <x:c r="F7" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add Friday management coverage from 08:00 to 18:10
</commit_message>
<xml_diff>
--- a/grafik-dyzurow-nadzoru-2026-2027.xlsx
+++ b/grafik-dyzurow-nadzoru-2026-2027.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="grafik" sheetId="1" r:id="Ra2e57b67bf9a48b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="numery telefonów" sheetId="2" r:id="R4ecf62a312224c2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="grafik" sheetId="1" r:id="R759bd946b214447e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="numery telefonów" sheetId="2" r:id="Rcbd0170340f14426"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -382,7 +382,9 @@
       <x:c r="E3" t="str">
         <x:v>Małgorzata Kończyńska</x:v>
       </x:c>
-      <x:c r="F3" t="str"/>
+      <x:c r="F3" t="str">
+        <x:v>Małgorzata Kończyńska</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
@@ -433,6 +435,18 @@
       <x:c r="D7" t="str"/>
       <x:c r="E7" t="str"/>
       <x:c r="F7" t="str"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>13:30 - 18:10</x:v>
+      </x:c>
+      <x:c r="B8"/>
+      <x:c r="C8"/>
+      <x:c r="D8"/>
+      <x:c r="E8"/>
+      <x:c r="F8" t="str">
+        <x:v>Arkadiusz Mocarski</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Split Friday morning management coverage at 09:30
</commit_message>
<xml_diff>
--- a/grafik-dyzurow-nadzoru-2026-2027.xlsx
+++ b/grafik-dyzurow-nadzoru-2026-2027.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="grafik" sheetId="1" r:id="R759bd946b214447e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="numery telefonów" sheetId="2" r:id="Rcbd0170340f14426"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="grafik" sheetId="1" r:id="R21a084e70d6049ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="numery telefonów" sheetId="2" r:id="R5528ff1d87244c07"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -382,9 +382,7 @@
       <x:c r="E3" t="str">
         <x:v>Małgorzata Kończyńska</x:v>
       </x:c>
-      <x:c r="F3" t="str">
-        <x:v>Małgorzata Kończyńska</x:v>
-      </x:c>
+      <x:c r="F3"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
@@ -446,6 +444,30 @@
       <x:c r="E8"/>
       <x:c r="F8" t="str">
         <x:v>Arkadiusz Mocarski</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>08:00 - 09:30</x:v>
+      </x:c>
+      <x:c r="B9"/>
+      <x:c r="C9"/>
+      <x:c r="D9"/>
+      <x:c r="E9"/>
+      <x:c r="F9" t="str">
+        <x:v>Małgorzata Kończyńska</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>09:30 - 13:30</x:v>
+      </x:c>
+      <x:c r="B10"/>
+      <x:c r="C10"/>
+      <x:c r="D10"/>
+      <x:c r="E10"/>
+      <x:c r="F10" t="str">
+        <x:v>Maciej Najwer</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Correct Friday handover times to 10:00 and 14:00
</commit_message>
<xml_diff>
--- a/grafik-dyzurow-nadzoru-2026-2027.xlsx
+++ b/grafik-dyzurow-nadzoru-2026-2027.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="grafik" sheetId="1" r:id="R21a084e70d6049ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="numery telefonów" sheetId="2" r:id="R5528ff1d87244c07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="grafik" sheetId="1" r:id="Rc4333c881c014947"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="numery telefonów" sheetId="2" r:id="Rd65a7dfa8510465f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -436,7 +436,7 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>13:30 - 18:10</x:v>
+        <x:v>14:00 - 18:10</x:v>
       </x:c>
       <x:c r="B8"/>
       <x:c r="C8"/>
@@ -448,7 +448,7 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>08:00 - 09:30</x:v>
+        <x:v>08:00 - 10:00</x:v>
       </x:c>
       <x:c r="B9"/>
       <x:c r="C9"/>
@@ -460,7 +460,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>09:30 - 13:30</x:v>
+        <x:v>10:00 - 14:00</x:v>
       </x:c>
       <x:c r="B10"/>
       <x:c r="C10"/>

</xml_diff>

<commit_message>
Popraw dyżury nadzoru na 24 i 25 września
Czwartek 24.09: popołudniowy dyżur przejmuje Małgorzata Kończyńska
w godzinach 13:30-18:10, zamiast Macieja Najwera do 19:00.

Piątek 25.09: po 13:30 nie ma dyżuru z powodu Święta Szkoły. Wiersz
popołudniowy znika z arkusza, a powód wchodzi do supervisionNotes, więc
strona pokazuje go jako uwagę przy piątku. Dyżur poranny 8:00-13:30
Małgorzaty Kończyńskiej zostaje bez zmian.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HKYjEPHLPESaJPNh8SzN51
</commit_message>
<xml_diff>
--- a/grafik-dyzurow-nadzoru-2026-2027.xlsx
+++ b/grafik-dyzurow-nadzoru-2026-2027.xlsx
@@ -329,7 +329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -423,30 +423,38 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>13:30 - 18:10</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Małgorzata Kończyńska</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>13:30 - 19:00</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr">
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
         <is>
           <t>Małgorzata Kończyńska</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Wiesław Filipiak</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Maciej Najwer</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Wiesław Filipiak</t>
-        </is>
-      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Popraw dyżur poranny 25 września
Piątkowy dyżur 8:00-13:30 obejmuje Marzena Filusz zamiast Małgorzaty
Kończyńskiej. Popołudnie bez zmian: Święto Szkoły, brak dyżuru.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HKYjEPHLPESaJPNh8SzN51
</commit_message>
<xml_diff>
--- a/grafik-dyzurow-nadzoru-2026-2027.xlsx
+++ b/grafik-dyzurow-nadzoru-2026-2027.xlsx
@@ -400,7 +400,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Małgorzata Kończyńska</t>
+          <t>Marzena Filusz</t>
         </is>
       </c>
     </row>
@@ -415,10 +415,6 @@
           <t>Wiesław Filipiak</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -426,15 +422,11 @@
           <t>13:30 - 18:10</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>Małgorzata Kończyńska</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -442,7 +434,6 @@
           <t>13:30 - 19:00</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>Małgorzata Kończyńska</t>
@@ -453,8 +444,6 @@
           <t>Wiesław Filipiak</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Dyżury nadzoru i pomoc p-p: widok całego tygodnia i wybór tygodnia
Grafik nadzoru trzyma każdy tydzień w osobnym arkuszu „grafik RRRR-MM-DD”
(data poniedziałku), więc poprzednie tygodnie zostają do wglądu. Dodany
tydzień 28.09–02.10.2026: wtorek rano do ustalenia, w środę rano Maciej
Najwer. Uwagi do dni (supervisionNotes) są teraz kluczowane datą, a zakres
obowiązywania wynika z arkuszy zamiast z supervisionValidFrom/To.

Strony dyżurów nadzoru i pomocy psychologiczno-pedagogicznej od 768 px
otwierają się na całym bieżącym tygodniu (w weekend — na nadchodzącym),
mają przyciski poprzedni/następny tydzień i powrót do bieżącego, a
nagłówki dni pokazują daty. Na telefonie domyślnie zostaje dzisiejszy dzień.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014QHcrFkQMT5XrsTLmHKX1m
</commit_message>
<xml_diff>
--- a/grafik-dyzurow-nadzoru-2026-2027.xlsx
+++ b/grafik-dyzurow-nadzoru-2026-2027.xlsx
@@ -3,8 +3,9 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="grafik" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="numery telefonów" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="grafik 2026-09-21" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="grafik 2026-09-28" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="numery telefonów" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -456,6 +457,121 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>godziny</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>poniedziałek</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>wtorek</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>środa</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>czwartek</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>piątek</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>08:00 - 13:30</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Maciej Najwer</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Maciej Najwer</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Marzena Filusz</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Małgorzata Kończyńska</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>13:30 - 19:00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Marzena Filusz</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Małgorzata Kończyńska</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Wiesław Filipiak</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Maciej Najwer</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Wiesław Filipiak</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Grafik nadzoru 28.09–02.10: podział zmian we wtorek i piątek
Wtorek rano: Maciej Najwer 8:00–9:00, Wiesław Filipiak 9:00–13:30.
Piątek: Maciej Najwer 8:00–10:00, Wiesław Filipiak 10:00–12:00,
Małgorzata Kończyńska 12:00–17:20. Znika uwaga „do ustalenia” z 29.09.

Komórka grafiku może teraz dzielić zmianę między osoby:
„Osoba A (8:00-9:00); Osoba B (9:00-13:30)” — godziny w nawiasie
zastępują godziny wiersza. Test importu i opis w README.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014QHcrFkQMT5XrsTLmHKX1m
</commit_message>
<xml_diff>
--- a/grafik-dyzurow-nadzoru-2026-2027.xlsx
+++ b/grafik-dyzurow-nadzoru-2026-2027.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -511,6 +511,11 @@
           <t>Maciej Najwer</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Maciej Najwer (8:00-9:00); Wiesław Filipiak (9:00-13:30)</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>Maciej Najwer</t>
@@ -523,7 +528,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Małgorzata Kończyńska</t>
+          <t>Maciej Najwer (8:00-10:00); Wiesław Filipiak (10:00-12:00)</t>
         </is>
       </c>
     </row>
@@ -555,12 +560,10 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Wiesław Filipiak</t>
-        </is>
-      </c>
-    </row>
-    <row r="4"/>
-    <row r="5"/>
+          <t>Małgorzata Kończyńska (12:00-17:20)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Grafik nadzoru 28.09–02.10: wtorek Kończyńska rano, Filusz po południu
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014QHcrFkQMT5XrsTLmHKX1m
</commit_message>
<xml_diff>
--- a/grafik-dyzurow-nadzoru-2026-2027.xlsx
+++ b/grafik-dyzurow-nadzoru-2026-2027.xlsx
@@ -513,7 +513,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Maciej Najwer (8:00-9:00); Wiesław Filipiak (9:00-13:30)</t>
+          <t>Małgorzata Kończyńska</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -545,7 +545,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Małgorzata Kończyńska</t>
+          <t>Marzena Filusz</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">

</xml_diff>

<commit_message>
Grafik nadzoru 02.10: Najwer 8:00–14:00, Kończyńska 14:00–17:20
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014QHcrFkQMT5XrsTLmHKX1m
</commit_message>
<xml_diff>
--- a/grafik-dyzurow-nadzoru-2026-2027.xlsx
+++ b/grafik-dyzurow-nadzoru-2026-2027.xlsx
@@ -528,7 +528,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Maciej Najwer</t>
+          <t>Maciej Najwer (8:00-14:00)</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Małgorzata Kończyńska (12:00-17:20)</t>
+          <t>Małgorzata Kończyńska (14:00-17:20)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Grafik nadzoru 05.10–09.10: wtorek i piątek po południu
Wtorek 06.10, 13:30–19:00: Wiesław Filipiak (zamiast Marzeny Filusz).
Piątek 09.10, 13:30–19:00: Arkadiusz Mocarski (zamiast Wiesława
Filipiaka). Pozostałe dni bez zmian.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014QHcrFkQMT5XrsTLmHKX1m
</commit_message>
<xml_diff>
--- a/grafik-dyzurow-nadzoru-2026-2027.xlsx
+++ b/grafik-dyzurow-nadzoru-2026-2027.xlsx
@@ -664,7 +664,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Marzena Filusz</t>
+          <t>Wiesław Filipiak</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -679,7 +679,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Wiesław Filipiak</t>
+          <t>Arkadiusz Mocarski</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Grafik nadzoru: zmiana popołudniowa kończy się z ostatnią lekcją
Dotąd tygodnie 28.09 i 05.10 miały popołudniowy dyżur do 19:00 we
wszystkie dni. Koniec zmiany wynika teraz z planu: ostatnia lekcja
oddziałów poza 1B i 3B (mają zajęcia wieczorne, do 19:50) kończy się
w pn i wt o 17:20, w śr o 16:30, w czw o 18:10, w pt o 17:20.

Dni z różnymi zakończeniami są osobnymi wierszami arkusza (jak w tygodniu
21.09). Osoby bez zmian. Reguła i godziny opisane w README.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014QHcrFkQMT5XrsTLmHKX1m
</commit_message>
<xml_diff>
--- a/grafik-dyzurow-nadzoru-2026-2027.xlsx
+++ b/grafik-dyzurow-nadzoru-2026-2027.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -536,7 +536,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>13:30 - 19:00</t>
+          <t>13:30 - 17:20</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -549,19 +549,33 @@
           <t>Marzena Filusz</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Małgorzata Kończyńska (14:00-17:20)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>13:30 - 16:30</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
         <is>
           <t>Wiesław Filipiak</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>13:30 - 18:10</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>Maciej Najwer</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Małgorzata Kończyńska (14:00-17:20)</t>
         </is>
       </c>
     </row>
@@ -576,7 +590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -654,7 +668,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>13:30 - 19:00</t>
+          <t>13:30 - 17:20</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -667,19 +681,33 @@
           <t>Wiesław Filipiak</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Arkadiusz Mocarski</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>13:30 - 16:30</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
         <is>
           <t>Wiesław Filipiak</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>13:30 - 18:10</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>Maciej Najwer</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Arkadiusz Mocarski</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Grafik nadzoru 12–16.10.2026: nowa obsada, środa 14.10 bez dyżuru
Wtorek 13.10: rano Małgorzata Kończyńska, po południu Wiesław Filipiak
(zamiast podziału Mocarski / Kończyńska od 13:00). Środa 14.10 (Dzień
Edukacji Narodowej, dzień wolny): bez dyżuru. Czwartek 15.10 rano Wiesław
Filipiak (zamiast Marzeny Filusz), piątek 16.10 po południu Arkadiusz
Mocarski (zamiast Wiesława Filipiaka).

Koniec zmiany popołudniowej z planu (ostatnia lekcja oddziałów poza 1B
i 3B): pn, wt, pt 17:20, czw 18:10. Tydzień 05.10 bez zmian.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014QHcrFkQMT5XrsTLmHKX1m
</commit_message>
<xml_diff>
--- a/grafik-dyzurow-nadzoru-2026-2027.xlsx
+++ b/grafik-dyzurow-nadzoru-2026-2027.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="grafik 2026-09-21" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="grafik 2026-09-28" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="grafik 2026-10-05" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="grafik 2026-10-12" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="numery telefonów" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="grafik 2026-09-21" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="grafik 2026-09-28" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="grafik 2026-10-05" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="grafik 2026-10-12" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="numery telefonów" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -723,7 +723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -779,17 +779,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Arkadiusz Mocarski (8:00-13:00)</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Arkadiusz Mocarski (8:00-13:00)</t>
+          <t>Małgorzata Kończyńska</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Marzena Filusz</t>
+          <t>Wiesław Filipiak</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -801,7 +796,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>13:30 - 19:00</t>
+          <t>13:30 - 17:20</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -811,22 +806,24 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Małgorzata Kończyńska (13:00-19:00)</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Wiesław Filipiak (13:00-19:00)</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
+          <t>Wiesław Filipiak</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Arkadiusz Mocarski</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>13:30 - 18:10</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>Maciej Najwer</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Wiesław Filipiak</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Grafik nadzoru 12–16.10: dyżur popołudniowy do 19:00
Na polecenie: w tygodniu 12–16.10 zmiana popołudniowa trwa 13:30–19:00
(pn, wt, czw, pt), zamiast końca wg planu lekcji. Obsada bez zmian,
środa 14.10 nadal bez dyżuru. Tygodnie 28.09 i 05.10 bez zmian.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014QHcrFkQMT5XrsTLmHKX1m
</commit_message>
<xml_diff>
--- a/grafik-dyzurow-nadzoru-2026-2027.xlsx
+++ b/grafik-dyzurow-nadzoru-2026-2027.xlsx
@@ -723,7 +723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -796,7 +796,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>13:30 - 17:20</t>
+          <t>13:30 - 19:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -809,21 +809,14 @@
           <t>Wiesław Filipiak</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Maciej Najwer</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>Arkadiusz Mocarski</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>13:30 - 18:10</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Maciej Najwer</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Grafik nadzoru 12–16.10: poprawka obsady
Wtorek 13.10: Arkadiusz Mocarski do 13:00, Małgorzata Kończyńska od
13:00 do 19:00. Środa 14.10 bez dyżuru (dzień wolny). Czwartek 15.10
rano Wiesław Filipiak, po południu Maciej Najwer. Piątek 16.10 rano
Małgorzata Kończyńska, po południu Wiesław Filipiak. Poniedziałek bez
zmian. Popołudnie do 19:00.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014QHcrFkQMT5XrsTLmHKX1m
</commit_message>
<xml_diff>
--- a/grafik-dyzurow-nadzoru-2026-2027.xlsx
+++ b/grafik-dyzurow-nadzoru-2026-2027.xlsx
@@ -779,7 +779,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Małgorzata Kończyńska</t>
+          <t>Arkadiusz Mocarski (8:00-13:00)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -806,17 +806,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Małgorzata Kończyńska (13:00-19:00)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Maciej Najwer</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>Wiesław Filipiak</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Maciej Najwer</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Arkadiusz Mocarski</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Grafik nadzoru 12–16.10: wtorek rano Najwer, środa z dyżurem, czwartek Filusz
Wtorek 13.10: Maciej Najwer do 13:00, Małgorzata Kończyńska od 13:00.
Środa 14.10: Arkadiusz Mocarski do 13:00, Wiesław Filipiak od 13:00.
Czwartek 15.10 rano Marzena Filusz, po południu Maciej Najwer. Poniedziałek
i piątek bez zmian. Popołudnie do 19:00. Tydzień 05.10 bez zmian.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014QHcrFkQMT5XrsTLmHKX1m
</commit_message>
<xml_diff>
--- a/grafik-dyzurow-nadzoru-2026-2027.xlsx
+++ b/grafik-dyzurow-nadzoru-2026-2027.xlsx
@@ -779,12 +779,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Maciej Najwer (8:00-13:00)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>Arkadiusz Mocarski (8:00-13:00)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Wiesław Filipiak</t>
+          <t>Marzena Filusz</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -807,6 +812,11 @@
       <c r="C3" t="inlineStr">
         <is>
           <t>Małgorzata Kończyńska (13:00-19:00)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Wiesław Filipiak (13:00-19:00)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">

</xml_diff>

<commit_message>
Grafik nadzoru 22–23.10: czwartek i piątek rano
Czwartek 22.10 rano Małgorzata Kończyńska (zamiast Marzeny Filusz),
piątek 23.10 rano Arkadiusz Mocarski (zamiast Małgorzaty Kończyńskiej).
Popołudnia i reszta tygodnia 19–23.10 bez zmian.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014QHcrFkQMT5XrsTLmHKX1m
</commit_message>
<xml_diff>
--- a/grafik-dyzurow-nadzoru-2026-2027.xlsx
+++ b/grafik-dyzurow-nadzoru-2026-2027.xlsx
@@ -908,12 +908,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Marzena Filusz</t>
+          <t>Małgorzata Kończyńska</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Małgorzata Kończyńska</t>
+          <t>Arkadiusz Mocarski</t>
         </is>
       </c>
     </row>

</xml_diff>